<commit_message>
Travail sur les consentements + corrections liés aux issues + revue du narratif + ajout d'un critère de recherche sur le statut de la préadmission pour le profil Encounter + ajout d'un capabilitystatement pour préciser les actions possibles sur les ressources 42f20bac468644407ee642d2f325d2f45519375f
</commit_message>
<xml_diff>
--- a/nmoreau/ig/StructureDefinition-appointment-context-extension.xlsx
+++ b/nmoreau/ig/StructureDefinition-appointment-context-extension.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-05-14T09:00:47+00:00</t>
+    <t>2025-05-22T16:12:30+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -132,7 +132,7 @@
     <t>Context</t>
   </si>
   <si>
-    <t>element:Element</t>
+    <t>element:Appointment</t>
   </si>
   <si>
     <t>ID</t>

</xml_diff>